<commit_message>
Add US and additional UK calendars
</commit_message>
<xml_diff>
--- a/tests/workbooks/test_calendars.xlsx
+++ b/tests/workbooks/test_calendars.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\tests\workbooks\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sebastian\01_GitHub\sschlenkrich\QuantLibXlOil\tests\workbooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6823EF69-2FA7-417C-B09F-FDA6AD3CCA6D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31892F8B-841E-4D0A-9182-E6DF240FA8E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" xr2:uid="{93E3CEBE-2A7E-45F9-A944-9E4960940BAD}"/>
+    <workbookView xWindow="6984" yWindow="-1032" windowWidth="30948" windowHeight="16728" xr2:uid="{93E3CEBE-2A7E-45F9-A944-9E4960940BAD}"/>
   </bookViews>
   <sheets>
     <sheet name="types" sheetId="1" r:id="rId1"/>
@@ -24,12 +24,26 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="83">
   <si>
     <t>ARGENTINA</t>
   </si>
@@ -263,6 +277,21 @@
   </si>
   <si>
     <t>qlCalender</t>
+  </si>
+  <si>
+    <t>UK_Settlement</t>
+  </si>
+  <si>
+    <t>UK_SETTLEMENT</t>
+  </si>
+  <si>
+    <t>US_SETTLEMENT</t>
+  </si>
+  <si>
+    <t>US_FEDERALRESERVE</t>
+  </si>
+  <si>
+    <t>US_SOFR</t>
   </si>
 </sst>
 </file>
@@ -278,18 +307,12 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -304,9 +327,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -314,7 +336,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -330,9 +352,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -370,7 +392,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -476,7 +498,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -618,7 +640,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -626,407 +648,450 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3075420B-A904-48C0-8CC0-21FB5C882A54}">
-  <dimension ref="B2:C45"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="B2:C50"/>
+  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="37.140625" customWidth="1"/>
+    <col min="2" max="2" width="37.109375" customWidth="1"/>
     <col min="3" max="3" width="27" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B2" t="s">
         <v>0</v>
       </c>
-      <c r="C2" t="e">
-        <f ca="1">_xll.qlCalendar(B2)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="3" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C2" t="str">
+        <f>_xll.qlCalendar(B2)</f>
+        <v>Buenos Aires stock exchange</v>
+      </c>
+    </row>
+    <row r="3" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
         <v>1</v>
       </c>
-      <c r="C3" t="e">
-        <f ca="1">_xll.qlCalendar(B3)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="4" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C3" t="str">
+        <f>_xll.qlCalendar(B3)</f>
+        <v>Australia settlement</v>
+      </c>
+    </row>
+    <row r="4" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B4" t="s">
         <v>2</v>
       </c>
-      <c r="C4" t="e">
-        <f ca="1">_xll.qlCalendar(B4)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="5" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C4" t="str">
+        <f>_xll.qlCalendar(B4)</f>
+        <v>Austrian settlement</v>
+      </c>
+    </row>
+    <row r="5" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B5" t="s">
         <v>3</v>
       </c>
-      <c r="C5" t="e">
-        <f ca="1">_xll.qlCalendar(B5)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="6" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C5" t="str">
+        <f>_xll.qlCalendar(B5)</f>
+        <v>Botswana</v>
+      </c>
+    </row>
+    <row r="6" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B6" t="s">
         <v>4</v>
       </c>
-      <c r="C6" t="e">
-        <f ca="1">_xll.qlCalendar(B6)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="7" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C6" t="str">
+        <f>_xll.qlCalendar(B6)</f>
+        <v>Brazil</v>
+      </c>
+    </row>
+    <row r="7" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B7" t="s">
         <v>5</v>
       </c>
-      <c r="C7" t="e">
-        <f ca="1">_xll.qlCalendar(B7)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="8" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C7" t="str">
+        <f>_xll.qlCalendar(B7)</f>
+        <v>Canada</v>
+      </c>
+    </row>
+    <row r="8" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B8" t="s">
         <v>6</v>
       </c>
-      <c r="C8" t="e">
-        <f ca="1">_xll.qlCalendar(B8)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="9" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C8" t="str">
+        <f>_xll.qlCalendar(B8)</f>
+        <v>Santiago Stock Exchange</v>
+      </c>
+    </row>
+    <row r="9" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B9" t="s">
         <v>7</v>
       </c>
-      <c r="C9" t="e">
-        <f ca="1">_xll.qlCalendar(B9)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="10" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C9" t="str">
+        <f>_xll.qlCalendar(B9)</f>
+        <v>Shanghai stock exchange</v>
+      </c>
+    </row>
+    <row r="10" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B10" t="s">
         <v>8</v>
       </c>
-      <c r="C10" t="e">
-        <f ca="1">_xll.qlCalendar(B10)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="11" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C10" t="str">
+        <f>_xll.qlCalendar(B10)</f>
+        <v>Prague stock exchange</v>
+      </c>
+    </row>
+    <row r="11" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B11" t="s">
         <v>9</v>
       </c>
-      <c r="C11" t="e">
-        <f ca="1">_xll.qlCalendar(B11)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="12" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C11" t="str">
+        <f>_xll.qlCalendar(B11)</f>
+        <v>Denmark</v>
+      </c>
+    </row>
+    <row r="12" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B12" t="s">
         <v>10</v>
       </c>
-      <c r="C12" t="e">
-        <f ca="1">_xll.qlCalendar(B12)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="13" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C12" t="str">
+        <f>_xll.qlCalendar(B12)</f>
+        <v>Finland</v>
+      </c>
+    </row>
+    <row r="13" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B13" t="s">
         <v>11</v>
       </c>
-      <c r="C13" t="e">
-        <f ca="1">_xll.qlCalendar(B13)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="14" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C13" t="str">
+        <f>_xll.qlCalendar(B13)</f>
+        <v>French settlement</v>
+      </c>
+    </row>
+    <row r="14" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B14" t="s">
         <v>12</v>
       </c>
-      <c r="C14" t="e">
-        <f ca="1">_xll.qlCalendar(B14)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="15" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C14" t="str">
+        <f>_xll.qlCalendar(B14)</f>
+        <v>Frankfurt stock exchange</v>
+      </c>
+    </row>
+    <row r="15" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B15" t="s">
         <v>13</v>
       </c>
-      <c r="C15" t="e">
-        <f ca="1">_xll.qlCalendar(B15)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="16" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C15" t="str">
+        <f>_xll.qlCalendar(B15)</f>
+        <v>Hong Kong stock exchange</v>
+      </c>
+    </row>
+    <row r="16" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B16" t="s">
         <v>14</v>
       </c>
-      <c r="C16" t="e">
-        <f ca="1">_xll.qlCalendar(B16)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="17" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C16" t="str">
+        <f>_xll.qlCalendar(B16)</f>
+        <v>Hungary</v>
+      </c>
+    </row>
+    <row r="17" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B17" t="s">
         <v>15</v>
       </c>
-      <c r="C17" t="e">
-        <f ca="1">_xll.qlCalendar(B17)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="18" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C17" t="str">
+        <f>_xll.qlCalendar(B17)</f>
+        <v>Iceland stock exchange</v>
+      </c>
+    </row>
+    <row r="18" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B18" t="s">
         <v>16</v>
       </c>
-      <c r="C18" t="e">
-        <f ca="1">_xll.qlCalendar(B18)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="19" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C18" t="str">
+        <f>_xll.qlCalendar(B18)</f>
+        <v>National Stock Exchange of India</v>
+      </c>
+    </row>
+    <row r="19" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B19" t="s">
         <v>17</v>
       </c>
-      <c r="C19" t="e">
-        <f ca="1">_xll.qlCalendar(B19)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="20" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C19" t="str">
+        <f>_xll.qlCalendar(B19)</f>
+        <v>Jakarta stock exchange</v>
+      </c>
+    </row>
+    <row r="20" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B20" t="s">
         <v>18</v>
       </c>
-      <c r="C20" t="e">
-        <f ca="1">_xll.qlCalendar(B20)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="21" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C20" t="str">
+        <f>_xll.qlCalendar(B20)</f>
+        <v>Tel Aviv stock exchange</v>
+      </c>
+    </row>
+    <row r="21" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B21" t="s">
         <v>19</v>
       </c>
-      <c r="C21" t="e">
-        <f ca="1">_xll.qlCalendar(B21)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="22" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C21" t="str">
+        <f>_xll.qlCalendar(B21)</f>
+        <v>Italian settlement</v>
+      </c>
+    </row>
+    <row r="22" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B22" t="s">
         <v>20</v>
       </c>
-      <c r="C22" t="e">
-        <f ca="1">_xll.qlCalendar(B22)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="23" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C22" t="str">
+        <f>_xll.qlCalendar(B22)</f>
+        <v>Japan</v>
+      </c>
+    </row>
+    <row r="23" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B23" t="s">
         <v>21</v>
       </c>
-      <c r="C23" t="e">
-        <f ca="1">_xll.qlCalendar(B23)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="24" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C23" t="str">
+        <f>_xll.qlCalendar(B23)</f>
+        <v>Mexican stock exchange</v>
+      </c>
+    </row>
+    <row r="24" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B24" t="s">
         <v>22</v>
       </c>
-      <c r="C24" t="e">
-        <f ca="1">_xll.qlCalendar(B24)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="25" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C24" t="str">
+        <f>_xll.qlCalendar(B24)</f>
+        <v>New Zealand (Wellington)</v>
+      </c>
+    </row>
+    <row r="25" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B25" t="s">
         <v>23</v>
       </c>
-      <c r="C25" t="e">
-        <f ca="1">_xll.qlCalendar(B25)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="26" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C25" t="str">
+        <f>_xll.qlCalendar(B25)</f>
+        <v>Norway</v>
+      </c>
+    </row>
+    <row r="26" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B26" t="s">
         <v>24</v>
       </c>
-      <c r="C26" t="e">
-        <f ca="1">_xll.qlCalendar(B26)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="27" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C26" t="str">
+        <f>_xll.qlCalendar(B26)</f>
+        <v>Poland Settlement</v>
+      </c>
+    </row>
+    <row r="27" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B27" t="s">
         <v>25</v>
       </c>
-      <c r="C27" t="e">
-        <f ca="1">_xll.qlCalendar(B27)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="28" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C27" t="str">
+        <f>_xll.qlCalendar(B27)</f>
+        <v>Bucharest stock exchange</v>
+      </c>
+    </row>
+    <row r="28" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B28" t="s">
         <v>26</v>
       </c>
-      <c r="C28" t="e">
-        <f ca="1">_xll.qlCalendar(B28)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="29" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C28" t="str">
+        <f>_xll.qlCalendar(B28)</f>
+        <v>Russian settlement</v>
+      </c>
+    </row>
+    <row r="29" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B29" t="s">
         <v>27</v>
       </c>
-      <c r="C29" t="e">
-        <f ca="1">_xll.qlCalendar(B29)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="30" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C29" t="str">
+        <f>_xll.qlCalendar(B29)</f>
+        <v>Tadawul</v>
+      </c>
+    </row>
+    <row r="30" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B30" t="s">
         <v>28</v>
       </c>
-      <c r="C30" t="e">
-        <f ca="1">_xll.qlCalendar(B30)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="31" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C30" t="str">
+        <f>_xll.qlCalendar(B30)</f>
+        <v>Singapore exchange</v>
+      </c>
+    </row>
+    <row r="31" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B31" t="s">
         <v>29</v>
       </c>
-      <c r="C31" t="e">
-        <f ca="1">_xll.qlCalendar(B31)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="32" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C31" t="str">
+        <f>_xll.qlCalendar(B31)</f>
+        <v>Bratislava stock exchange</v>
+      </c>
+    </row>
+    <row r="32" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B32" t="s">
         <v>30</v>
       </c>
-      <c r="C32" t="e">
-        <f ca="1">_xll.qlCalendar(B32)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="33" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C32" t="str">
+        <f>_xll.qlCalendar(B32)</f>
+        <v>South Africa</v>
+      </c>
+    </row>
+    <row r="33" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B33" t="s">
         <v>31</v>
       </c>
-      <c r="C33" t="e">
-        <f ca="1">_xll.qlCalendar(B33)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="34" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C33" t="str">
+        <f>_xll.qlCalendar(B33)</f>
+        <v>South-Korea exchange</v>
+      </c>
+    </row>
+    <row r="34" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B34" t="s">
         <v>32</v>
       </c>
-      <c r="C34" t="e">
-        <f ca="1">_xll.qlCalendar(B34)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="35" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C34" t="str">
+        <f>_xll.qlCalendar(B34)</f>
+        <v>Sweden</v>
+      </c>
+    </row>
+    <row r="35" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B35" t="s">
         <v>33</v>
       </c>
-      <c r="C35" t="e">
-        <f ca="1">_xll.qlCalendar(B35)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="36" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C35" t="str">
+        <f>_xll.qlCalendar(B35)</f>
+        <v>Switzerland</v>
+      </c>
+    </row>
+    <row r="36" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B36" t="s">
         <v>34</v>
       </c>
-      <c r="C36" t="e">
-        <f ca="1">_xll.qlCalendar(B36)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="37" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C36" t="str">
+        <f>_xll.qlCalendar(B36)</f>
+        <v>Taiwan stock exchange</v>
+      </c>
+    </row>
+    <row r="37" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B37" t="s">
         <v>35</v>
       </c>
-      <c r="C37" t="e">
-        <f ca="1">_xll.qlCalendar(B37)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="38" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C37" t="str">
+        <f>_xll.qlCalendar(B37)</f>
+        <v>TARGET</v>
+      </c>
+    </row>
+    <row r="38" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B38" t="s">
         <v>36</v>
       </c>
-      <c r="C38" t="e">
-        <f ca="1">_xll.qlCalendar(B38)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="39" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C38" t="str">
+        <f>_xll.qlCalendar(B38)</f>
+        <v>Thailand stock exchange</v>
+      </c>
+    </row>
+    <row r="39" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B39" t="s">
         <v>37</v>
       </c>
-      <c r="C39" t="e">
-        <f ca="1">_xll.qlCalendar(B39)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="40" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C39" t="str">
+        <f>_xll.qlCalendar(B39)</f>
+        <v>Turkey</v>
+      </c>
+    </row>
+    <row r="40" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B40" t="s">
         <v>38</v>
       </c>
-      <c r="C40" t="e">
-        <f ca="1">_xll.qlCalendar(B40)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="41" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B41" s="1" t="s">
+      <c r="C40" t="str">
+        <f>_xll.qlCalendar(B40)</f>
+        <v>Ukrainian stock exchange</v>
+      </c>
+    </row>
+    <row r="41" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B41" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="C41" t="e">
-        <f ca="1">_xll.qlCalendar(B41)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="42" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C41" t="str">
+        <f>_xll.qlCalendar(B41)</f>
+        <v>New York stock exchange</v>
+      </c>
+    </row>
+    <row r="42" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B42" t="s">
         <v>40</v>
       </c>
-      <c r="C42" t="e">
-        <f ca="1">_xll.qlCalendar(B42)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="43" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C42" t="str">
+        <f>_xll.qlCalendar(B42)</f>
+        <v>UK settlement</v>
+      </c>
+    </row>
+    <row r="43" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B43" t="s">
         <v>41</v>
       </c>
-      <c r="C43" t="e">
-        <f ca="1">_xll.qlCalendar(B43)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="44" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C43" t="str">
+        <f>_xll.qlCalendar(B43)</f>
+        <v>Null</v>
+      </c>
+    </row>
+    <row r="44" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B44" t="s">
         <v>42</v>
       </c>
-      <c r="C44" t="e">
-        <f ca="1">_xll.qlCalendar(B44)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="45" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C44" t="str">
+        <f>_xll.qlCalendar(B44)</f>
+        <v>weekends only</v>
+      </c>
+    </row>
+    <row r="45" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B45" t="s">
         <v>43</v>
       </c>
-      <c r="C45" t="e">
-        <f ca="1">_xll.qlCalendar(B45)</f>
-        <v>#VALUE!</v>
+      <c r="C45" t="str">
+        <f>_xll.qlCalendar(B45)</f>
+        <v xml:space="preserve">ValueError: ValueError: Unknown calendar: UNKNOWN_KEY
+Traceback (most recent call last):
+  File "C:\Users\Sebastian\01_GitHub\sschlenkrich\QuantLibXlOil\src\quantlib_xloil\calendars.py", line 152, in qlCalendar
+    return _qCalendar(calendar_name)
+  File "C:\Users\Sebastian\01_GitHub\sschlenkrich\QuantLibXlOil\src\quantlib_xloil\calendars.py", line 117, in _qCalendar
+    raise ValueError(f"Unknown calendar: {name}")
+ValueError: Unknown calendar: UNKNOWN_KEY
+</v>
+      </c>
+    </row>
+    <row r="47" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B47" t="s">
+        <v>79</v>
+      </c>
+      <c r="C47" t="str">
+        <f>_xll.qlCalendar(B47)</f>
+        <v>UK settlement</v>
+      </c>
+    </row>
+    <row r="48" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B48" t="s">
+        <v>80</v>
+      </c>
+      <c r="C48" t="str">
+        <f>_xll.qlCalendar(B48)</f>
+        <v>US settlement</v>
+      </c>
+    </row>
+    <row r="49" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B49" t="s">
+        <v>81</v>
+      </c>
+      <c r="C49" t="str">
+        <f>_xll.qlCalendar(B49)</f>
+        <v>Federal Reserve Bankwire System</v>
+      </c>
+    </row>
+    <row r="50" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B50" t="s">
+        <v>82</v>
+      </c>
+      <c r="C50" t="str">
+        <f>_xll.qlCalendar(B50)</f>
+        <v>SOFR fixing calendar</v>
       </c>
     </row>
   </sheetData>
@@ -1038,222 +1103,215 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33850488-5007-411C-8F3E-026395460888}">
   <dimension ref="A1:E25"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="32.7109375" customWidth="1"/>
-    <col min="2" max="2" width="21.5703125" customWidth="1"/>
+    <col min="1" max="1" width="32.6640625" customWidth="1"/>
+    <col min="2" max="2" width="21.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>59</v>
       </c>
-      <c r="B1" t="e">
-        <f ca="1">_xll.qlCalendar("TARGET")</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B1" t="str">
+        <f>_xll.qlCalendar("TARGET")</f>
+        <v>TARGET</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>62</v>
       </c>
-      <c r="B2" s="2">
+      <c r="B2" s="1">
         <v>46171</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>65</v>
       </c>
-      <c r="B3" t="e">
-        <f ca="1">_xll.qlDateWeekday(B2)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B3" t="str">
+        <f>_xll.qlDateWeekday(B2)</f>
+        <v>FRIDAY</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>60</v>
       </c>
-      <c r="B4" s="2">
+      <c r="B4" s="1">
         <v>46023</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>61</v>
       </c>
-      <c r="B5" s="2">
+      <c r="B5" s="1">
         <v>46027</v>
       </c>
-      <c r="D5" s="2">
+      <c r="D5" s="1">
         <v>46025</v>
       </c>
-      <c r="E5" t="e">
-        <f ca="1">_xll.qlCalendarIsBusinessDay(B1,D5)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="E6" t="e">
-        <f ca="1">_xll.qlCalendarIsHoliday(B1,D5)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E5" t="b">
+        <f>_xll.qlCalendarIsBusinessDay(B1,D5)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E6" t="b">
+        <f>_xll.qlCalendarIsHoliday(B1,D5)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>44</v>
       </c>
-      <c r="B7" t="e">
-        <f ca="1">_xll.qlCalendarisWeekend($B$1,B3)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B7" t="b">
+        <f>_xll.qlCalendarisWeekend($B$1,B3)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>45</v>
       </c>
-      <c r="B8" s="2" t="e">
-        <f ca="1">_xll.qlCalendarStartOfMonth(B1,B2)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B8" s="1">
+        <f>_xll.qlCalendarStartOfMonth(B1,B2)</f>
+        <v>46146</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>46</v>
       </c>
-      <c r="B9" s="2" t="e">
-        <f ca="1">_xll.qlCalendarEndOfMonth(B1,B2)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B9" s="1">
+        <f>_xll.qlCalendarEndOfMonth(B1,B2)</f>
+        <v>46171</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>47</v>
       </c>
-      <c r="B10" t="e">
-        <f ca="1">_xll.qlCalendarIsBusinessDay(B1,B2)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B10" t="b">
+        <f>_xll.qlCalendarIsBusinessDay(B1,B2)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>48</v>
       </c>
-      <c r="B11" t="e">
-        <f ca="1">_xll.qlCalendarIsHoliday(B1,B2)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B11" t="b">
+        <f>_xll.qlCalendarIsHoliday(B1,B2)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>49</v>
       </c>
-      <c r="B12" t="e">
-        <f ca="1">_xll.qlCalendarIsEndOfMonth(B1,B2)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B12" t="b">
+        <f>_xll.qlCalendarIsEndOfMonth(B1,B2)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>50</v>
       </c>
-      <c r="B13" t="e">
-        <f ca="1">_xll.qlCalendarIsStartOfMonth(B1,B2)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B13" t="b">
+        <f>_xll.qlCalendarIsStartOfMonth(B1,B2)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>54</v>
       </c>
-      <c r="B14" t="e">
-        <f ca="1">_xll.qlCalendarBusinessDaysBetween(B1,B4,B5)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" s="3" t="s">
+      <c r="B14">
+        <f>_xll.qlCalendarBusinessDaysBetween(B1,B4,B5)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A15" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="B15" t="e">
-        <f ca="1">_xll.qlCalendarName(B1)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" s="3" t="s">
+      <c r="B15" t="str">
+        <f>_xll.qlCalendarName(B1)</f>
+        <v>TARGET</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A16" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B16" t="e">
-        <f ca="1">_xll.qlCalendarEmpty(B1)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" s="4" t="s">
+      <c r="B16" t="b">
+        <f>_xll.qlCalendarEmpty(B1)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A17" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="B17" s="2" t="e">
-        <f t="array" aca="1" ref="B17:B20" ca="1">_xll.qlCalendarHolidayList(B1,B4,B5)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" s="4"/>
-      <c r="B18" s="2" t="e">
-        <f ca="1"/>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" s="4"/>
-      <c r="B19" s="2" t="e">
-        <f ca="1"/>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" s="4"/>
-      <c r="B20" s="2" t="e">
-        <f ca="1"/>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21" s="4" t="s">
+      <c r="B17" s="1">
+        <f t="array" ref="B17:B20">_xll.qlCalendarHolidayList(B1,B4,B5)</f>
+        <v>46023</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A18" s="3"/>
+      <c r="B18" s="1">
+        <v>46024</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A19" s="3"/>
+      <c r="B19" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A20" s="3"/>
+      <c r="B20" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A21" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="B21" s="2" t="e">
-        <f t="array" aca="1" ref="B21:B25" ca="1">_xll.qlCalendarBusinessDayList(B1,B4,B5)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22" s="4"/>
-      <c r="B22" s="2" t="e">
-        <f ca="1"/>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A23" s="4"/>
-      <c r="B23" t="e">
-        <f ca="1"/>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A24" s="4"/>
-      <c r="B24" t="e">
-        <f ca="1"/>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A25" s="4"/>
-      <c r="B25" t="e">
-        <f ca="1"/>
-        <v>#VALUE!</v>
+      <c r="B21" s="1">
+        <f t="array" ref="B21:B25">_xll.qlCalendarBusinessDayList(B1,B4,B5)</f>
+        <v>46027</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A22" s="3"/>
+      <c r="B22" s="1">
+        <v>46027</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A23" s="3"/>
+      <c r="B23">
+        <v>46027</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A24" s="3"/>
+      <c r="B24">
+        <v>46027</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A25" s="3"/>
+      <c r="B25">
+        <v>46027</v>
       </c>
     </row>
   </sheetData>
@@ -1269,140 +1327,134 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{41849B37-CA87-4E4A-8B76-B839138C7508}">
   <dimension ref="A2:B23"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="46.42578125" customWidth="1"/>
+    <col min="1" max="1" width="46.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>59</v>
       </c>
-      <c r="B2" t="e">
-        <f ca="1">_xll.qlCalendar("TARGET")</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B2" t="str">
+        <f>_xll.qlCalendar("TARGET")</f>
+        <v>TARGET</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>63</v>
       </c>
-      <c r="B3" s="2">
+      <c r="B3" s="1">
         <v>46024</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>64</v>
       </c>
-      <c r="B4" s="2">
+      <c r="B4" s="1">
         <v>46023</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>60</v>
       </c>
-      <c r="B5" s="2">
+      <c r="B5" s="1">
         <v>46023</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>61</v>
       </c>
-      <c r="B6" s="2">
+      <c r="B6" s="1">
         <v>46027</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>51</v>
       </c>
       <c r="B9" t="e">
-        <f ca="1">_xll.qlCalendarAddHoliday(B2,B3)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+        <f>_xll.qlCalendarAddHoliday(B2,B3)</f>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>55</v>
       </c>
-      <c r="B10" s="2" t="e">
-        <f t="array" aca="1" ref="B10:B12" ca="1">_xll.qlCalendarHolidayList(B2,B5,B6)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B11" s="2" t="e">
-        <f ca="1"/>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B12" s="2" t="e">
-        <f ca="1"/>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B10" s="1">
+        <f t="array" ref="B10:B12">_xll.qlCalendarHolidayList(B2,B5,B6)</f>
+        <v>46023</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B11" s="1">
+        <v>46024</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B12" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>52</v>
       </c>
       <c r="B14" t="e">
-        <f ca="1">_xll.qlCalendarRemoveHoliday(B2,B4)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+        <f>_xll.qlCalendarRemoveHoliday(B2,B4)</f>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>55</v>
       </c>
-      <c r="B15" s="2" t="e">
-        <f t="array" aca="1" ref="B15:B17" ca="1">_xll.qlCalendarHolidayList(B2,B5,B6)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B16" s="2" t="e">
-        <f ca="1"/>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B17" s="2" t="e">
-        <f ca="1"/>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B15" s="1">
+        <f t="array" ref="B15:B17">_xll.qlCalendarHolidayList(B2,B5,B6)</f>
+        <v>46023</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B16" s="1">
+        <v>46023</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B17" s="1">
+        <v>46023</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>53</v>
       </c>
       <c r="B20" t="e">
-        <f ca="1">_xll.qlCalendarResetAddedAndRemovedHolidays(B2)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+        <f>_xll.qlCalendarResetAddedAndRemovedHolidays(B2)</f>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>55</v>
       </c>
-      <c r="B21" s="2" t="e">
-        <f t="array" aca="1" ref="B21:B23" ca="1">_xll.qlCalendarHolidayList(B2,B5,B6)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B22" s="2" t="e">
-        <f ca="1"/>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B23" s="2" t="e">
-        <f ca="1"/>
-        <v>#VALUE!</v>
+      <c r="B21" s="1">
+        <f t="array" ref="B21:B23">_xll.qlCalendarHolidayList(B2,B5,B6)</f>
+        <v>46023</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B22" s="1">
+        <v>46023</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B23" s="1">
+        <v>46023</v>
       </c>
     </row>
   </sheetData>
@@ -1413,30 +1465,30 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{92C2F300-0ACE-414A-85D4-FE4A0E362995}">
   <dimension ref="A1:C10"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
-    <col min="3" max="3" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>59</v>
       </c>
-      <c r="B1" t="e">
-        <f ca="1">_xll.qlCalendar("TARGET")</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B1" t="str">
+        <f>_xll.qlCalendar("TARGET")</f>
+        <v>TARGET</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>62</v>
       </c>
-      <c r="B2" s="2">
+      <c r="B2" s="1">
         <v>46053</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>74</v>
       </c>
@@ -1444,7 +1496,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>67</v>
       </c>
@@ -1452,16 +1504,16 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>68</v>
       </c>
       <c r="B5" t="s">
         <v>71</v>
       </c>
-      <c r="C5" s="2"/>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C5" s="1"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>69</v>
       </c>
@@ -1469,31 +1521,31 @@
         <v>70</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>72</v>
       </c>
-      <c r="B8" s="2" t="e">
-        <f ca="1">_xll.qlCalendarAdjust(B1,B2)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B8" s="1">
+        <f>_xll.qlCalendarAdjust(B1,B2)</f>
+        <v>46055</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>73</v>
       </c>
-      <c r="B9" s="2" t="e">
-        <f ca="1">_xll.qlCalendarAdvance(B1,B2,B4,B5,B3,1)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B9" s="1">
+        <f>_xll.qlCalendarAdvance(B1,B2,B4,B5,B3,1)</f>
+        <v>46066</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>73</v>
       </c>
-      <c r="B10" s="2" t="e">
-        <f ca="1">_xll.qlCalendarAdvance2(B1,B2,B6,B3,0)</f>
-        <v>#VALUE!</v>
+      <c r="B10" s="1">
+        <f>_xll.qlCalendarAdvance2(B1,B2,B6,B3,0)</f>
+        <v>46142</v>
       </c>
     </row>
   </sheetData>
@@ -1504,40 +1556,39 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DFBBB7C2-660D-4F66-9443-9DB0EA674324}">
   <dimension ref="A3:B8"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="22.7109375" customWidth="1"/>
-    <col min="2" max="2" width="49.85546875" customWidth="1"/>
+    <col min="1" max="1" width="22.6640625" customWidth="1"/>
+    <col min="2" max="2" width="49.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>59</v>
       </c>
-      <c r="B3" t="e">
-        <f ca="1">_xll.qlCalendar("Sweden")</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B3" t="str">
+        <f>_xll.qlCalendar("Sweden")</f>
+        <v>Sweden</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>59</v>
       </c>
-      <c r="B4" t="e">
-        <f ca="1">_xll.qlCalendar("TARGET")</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B4" t="str">
+        <f>_xll.qlCalendar("TARGET")</f>
+        <v>TARGET</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>77</v>
       </c>
-      <c r="B5" t="e">
-        <f ca="1">_xll.qlCalendar("UnitedKingdom")</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B5" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>75</v>
       </c>
@@ -1545,16 +1596,16 @@
         <v>76</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B7" t="e">
-        <f ca="1">_xll.qlCalendarJointCalendar(B3,B4,B6)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B8" t="e">
-        <f ca="1">_xll.qlCalendarJointCalendar2(B3,B4,B5)</f>
-        <v>#VALUE!</v>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B7" t="str">
+        <f>_xll.qlCalendarJointCalendar(B3,B4,B6)</f>
+        <v>JoinHolidays(Sweden, TARGET)</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B8" t="str">
+        <f>_xll.qlCalendarJointCalendar2(B3,B4,B5)</f>
+        <v>JoinHolidays(Sweden, TARGET, UK settlement)</v>
       </c>
     </row>
   </sheetData>

</xml_diff>